<commit_message>
fix: phonetic runs and out-of-range anchors in workbook comments
Ruby readings (<rPh>) no longer leak into legacy note bodies, and a
comment anchored past the used range grows the grid — its corner
tint is visible and the cursor can reach it, like formula-only
cells. Both were confirmed by the (interrupted) adversarial pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYXhWAPZoQiTpduL3XFCVJ
</commit_message>
<xml_diff>
--- a/tests/fixtures/comments.xlsx
+++ b/tests/fixtures/comments.xlsx
@@ -18,8 +18,18 @@
         <r>
           <t>昔のメモ</t>
         </r>
+        <rPh sb="0" eb="2">
+          <t>ムカシ</t>
+        </rPh>
         <r>
           <t>の続き</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D9" authorId="9">
+      <text>
+        <r>
+          <t>範囲外のメモ</t>
         </r>
       </text>
     </comment>

</xml_diff>